<commit_message>
Move registration application to phase four
</commit_message>
<xml_diff>
--- a/outputs/reeds_checklist/睿思實驗教育機構_115-116籌備工作檢核表.xlsx
+++ b/outputs/reeds_checklist/睿思實驗教育機構_115-116籌備工作檢核表.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="Rb4ef45bc917d43c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="階段總覽" sheetId="2" r:id="R439d619fbbec4653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作檢核表" sheetId="3" r:id="R234ab1b36545430c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修正紀錄" sheetId="4" r:id="Rc446401012e44596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始計畫摘要" sheetId="5" r:id="Rfa4690ff7fd74767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="清單" sheetId="6" r:id="Re671125a8a4a41e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用說明" sheetId="1" r:id="R7a7b87c14b9e434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="階段總覽" sheetId="2" r:id="Rd373fdb0a5c545bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作檢核表" sheetId="3" r:id="R0da20e1eb9114df4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修正紀錄" sheetId="4" r:id="Ra3cd242705a54d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始計畫摘要" sheetId="5" r:id="Rc652531b4e8c4f9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="清單" sheetId="6" r:id="R4b3fa4afd9ae497e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -441,12 +441,12 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{FD8D91D2-31E7-4230-9188-98CC2901B88D}"/>
+  <xltc:person displayName="User" id="{317B4F2F-5E1F-4AAE-BE94-1D60FD7C27E3}"/>
 </xltc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PrepChecklist" displayName="PrepChecklist" ref="A1:N42" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PrepChecklist" displayName="PrepChecklist" ref="A1:N42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="階段"/>
@@ -463,12 +463,12 @@
     <x:tableColumn id="13" name="風險/需修正事項"/>
     <x:tableColumn id="14" name="修正紀錄/下一步"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionLog" displayName="RevisionLog" ref="A1:I21" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RevisionLog" displayName="RevisionLog" ref="A1:I21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="日期"/>
     <x:tableColumn id="2" name="階段"/>
@@ -480,19 +480,19 @@
     <x:tableColumn id="8" name="追蹤期限"/>
     <x:tableColumn id="9" name="結案狀態"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceSummary" displayName="SourceSummary" ref="A1:D9" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceSummary" displayName="SourceSummary" ref="A1:D9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="階段"/>
     <x:tableColumn id="2" name="期程"/>
     <x:tableColumn id="3" name="主題"/>
     <x:tableColumn id="4" name="原始計畫重點摘要"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -539,9 +539,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1056,14 +1056,14 @@
         <x:v>115年12月-116年1月</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
-        <x:v>寒假試辦與培訓啟動期</x:v>
+        <x:v>寒假試辦、培訓啟動與立案申請期</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>透過營隊測試課程、新進師資共識培訓、硬體完工</x:v>
+        <x:v>透過營隊測試課程、新進師資共識培訓、硬體完工，並於12月15日前遞交正式立案申請</x:v>
       </x:c>
       <x:c r="E7" s="24" t="n">
         <x:f>COUNTIF('工作檢核表'!$B$2:$B$200,A7)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F7" s="24" t="n">
         <x:f>COUNTIFS('工作檢核表'!$B$2:$B$200,A7,'工作檢核表'!$K$2:$K$200,"已完成")</x:f>
@@ -1086,14 +1086,14 @@
         <x:v>116年2月-3月</x:v>
       </x:c>
       <x:c r="C8" s="24" t="str">
-        <x:v>機構立案與正式招生期</x:v>
+        <x:v>立案追蹤與正式招生期</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>遞交立案申請、全面啟動招生作業、設備進駐</x:v>
+        <x:v>追蹤立案補件、會勘與審查進度，全面啟動招生作業、設備進駐</x:v>
       </x:c>
       <x:c r="E8" s="24" t="n">
         <x:f>COUNTIF('工作檢核表'!$B$2:$B$200,A8)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="24" t="n">
         <x:f>COUNTIFS('工作檢核表'!$B$2:$B$200,A8,'工作檢核表'!$K$2:$K$200,"已完成")</x:f>
@@ -1299,7 +1299,7 @@
         <x:v>計畫主持人/行政籌備</x:v>
       </x:c>
       <x:c r="J2" s="54" t="n">
-        <x:v>46234</x:v>
+        <x:v>46198</x:v>
       </x:c>
       <x:c r="K2" s="46" t="str">
         <x:v>待開始</x:v>
@@ -1337,7 +1337,7 @@
         <x:v>計畫主持人/教務籌備</x:v>
       </x:c>
       <x:c r="J3" s="55" t="n">
-        <x:v>46234</x:v>
+        <x:v>46203</x:v>
       </x:c>
       <x:c r="K3" s="49" t="str">
         <x:v>待開始</x:v>
@@ -2263,10 +2263,10 @@
         <x:v>P5-01</x:v>
       </x:c>
       <x:c r="B28" s="49" t="str">
-        <x:v>第五期</x:v>
+        <x:v>第四期</x:v>
       </x:c>
       <x:c r="C28" s="49" t="str">
-        <x:v>116年2月-3月</x:v>
+        <x:v>115年12月-116年1月</x:v>
       </x:c>
       <x:c r="D28" s="49" t="str">
         <x:v>立案申請</x:v>
@@ -2287,7 +2287,7 @@
         <x:v>行政籌備</x:v>
       </x:c>
       <x:c r="J28" s="55" t="n">
-        <x:v>46477</x:v>
+        <x:v>46371</x:v>
       </x:c>
       <x:c r="K28" s="49" t="str">
         <x:v>待開始</x:v>
@@ -2848,7 +2848,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f888f34842d46b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd0d2dbcb334ed9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3125,7 +3125,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04954267d8e542e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15568925fbaf4cf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3204,10 +3204,10 @@
         <x:v>115年12月-116年1月</x:v>
       </x:c>
       <x:c r="C5" s="49" t="str">
-        <x:v>寒假試辦與培訓啟動期</x:v>
+        <x:v>寒假試辦、培訓啟動與立案申請期</x:v>
       </x:c>
       <x:c r="D5" s="50" t="str">
-        <x:v>透過營隊測試課程、新進師資共識培訓、硬體完工</x:v>
+        <x:v>透過營隊測試課程、新進師資共識培訓、硬體完工，並於12月15日前遞交正式立案申請</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3218,10 +3218,10 @@
         <x:v>116年2月-3月</x:v>
       </x:c>
       <x:c r="C6" s="49" t="str">
-        <x:v>機構立案與正式招生期</x:v>
+        <x:v>立案追蹤與正式招生期</x:v>
       </x:c>
       <x:c r="D6" s="50" t="str">
-        <x:v>遞交立案申請、全面啟動招生作業、設備進駐</x:v>
+        <x:v>追蹤立案補件、會勘與審查進度，全面啟動招生作業、設備進駐</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3269,7 +3269,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10df6dc6900f44f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c1ffd79de854335"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>